<commit_message>
feat(reconciliation): implement debt and finance models, routers and services
</commit_message>
<xml_diff>
--- a/ktx-backend/sample_statements/sao_ke_tien_phong_t9_tpbank.xlsx
+++ b/ktx-backend/sample_statements/sao_ke_tien_phong_t9_tpbank.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sao ke Thang 9" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,12 +459,14 @@
           <t>2026-09-12 10:00:00</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>600000</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>350000</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DTC245180037 nop tien phong</t>
+          <t>TP DTC245180037</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -489,8 +491,10 @@
           <t>2026-09-12 09:15:00</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>1800000</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>350000</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>

</xml_diff>